<commit_message>
Update workbook, add illustrative labels
</commit_message>
<xml_diff>
--- a/tangy_stitch_data.xlsx
+++ b/tangy_stitch_data.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="267">
   <si>
     <t xml:space="preserve">Fabric ID </t>
   </si>
@@ -463,6 +463,9 @@
     <t>Demo Supplier 09</t>
   </si>
   <si>
+    <t>TS-F031</t>
+  </si>
+  <si>
     <t>Sunday Monday</t>
   </si>
   <si>
@@ -472,13 +475,19 @@
     <t>Demo Supplier 10</t>
   </si>
   <si>
+    <t>TS-F032</t>
+  </si>
+  <si>
+    <t>TS-F033</t>
+  </si>
+  <si>
     <t>Double Georgette</t>
   </si>
   <si>
     <t>Olive</t>
   </si>
   <si>
-    <t>TS-F031</t>
+    <t>TS-F034</t>
   </si>
   <si>
     <t>Dark Purple</t>
@@ -2605,8 +2614,8 @@
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
-      <c r="A32" s="2" t="s">
-        <v>143</v>
+      <c r="A32" s="4" t="s">
+        <v>148</v>
       </c>
       <c r="B32" s="2">
         <v>540710.0</v>
@@ -2615,19 +2624,19 @@
         <v>540710.0</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>102</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G32" s="2" t="s">
         <v>42</v>
       </c>
       <c r="J32" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="K32" s="2" t="s">
         <v>25</v>
@@ -2652,8 +2661,8 @@
       </c>
     </row>
     <row r="33" ht="15.75" customHeight="1">
-      <c r="A33" s="2" t="s">
-        <v>143</v>
+      <c r="A33" s="4" t="s">
+        <v>152</v>
       </c>
       <c r="B33" s="2">
         <v>540710.0</v>
@@ -2668,13 +2677,13 @@
         <v>45</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G33" s="2" t="s">
         <v>42</v>
       </c>
       <c r="J33" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="K33" s="2" t="s">
         <v>25</v>
@@ -2699,8 +2708,8 @@
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
-      <c r="A34" s="2" t="s">
-        <v>143</v>
+      <c r="A34" s="4" t="s">
+        <v>153</v>
       </c>
       <c r="B34" s="2">
         <v>540710.0</v>
@@ -2709,19 +2718,19 @@
         <v>540710.0</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="G34" s="2" t="s">
         <v>42</v>
       </c>
       <c r="J34" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="K34" s="2" t="s">
         <v>25</v>
@@ -2746,8 +2755,8 @@
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
-      <c r="A35" s="2" t="s">
-        <v>153</v>
+      <c r="A35" s="4" t="s">
+        <v>156</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>76</v>
@@ -2756,13 +2765,13 @@
         <v>40</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="G35" s="2" t="s">
         <v>42</v>
       </c>
       <c r="J35" s="2" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="M35" s="2">
         <v>144.0</v>
@@ -3765,10 +3774,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>9</v>
@@ -3777,16 +3786,16 @@
         <v>11</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>16</v>
@@ -3797,10 +3806,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>24</v>
@@ -3809,7 +3818,7 @@
         <v>46256.0</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="F2" s="2">
         <v>1.041666667</v>
@@ -3829,10 +3838,10 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>24</v>
@@ -3841,7 +3850,7 @@
         <v>46256.0</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="F3" s="2">
         <v>1.041666666666667</v>
@@ -3861,10 +3870,10 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>163</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>24</v>
@@ -3873,7 +3882,7 @@
         <v>46256.0</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="F4" s="2">
         <v>1.736111111111111</v>
@@ -3893,10 +3902,10 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>24</v>
@@ -3905,7 +3914,7 @@
         <v>46256.0</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="F5" s="2">
         <v>1.041666666666667</v>
@@ -3925,10 +3934,10 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>24</v>
@@ -3937,7 +3946,7 @@
         <v>46256.0</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="F6" s="2">
         <v>1.388888888888889</v>
@@ -3957,10 +3966,10 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>24</v>
@@ -3969,7 +3978,7 @@
         <v>46256.0</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="F7" s="2">
         <v>1.041666666666667</v>
@@ -3989,10 +3998,10 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>24</v>
@@ -4001,7 +4010,7 @@
         <v>46256.0</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="F8" s="2">
         <v>1.736111111111111</v>
@@ -4021,10 +4030,10 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>55</v>
@@ -4033,7 +4042,7 @@
         <v>46256.0</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="F9" s="2">
         <v>1.25</v>
@@ -4053,10 +4062,10 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>66</v>
@@ -4065,7 +4074,7 @@
         <v>46256.0</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="F10" s="2">
         <v>1.0</v>
@@ -4085,10 +4094,10 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>66</v>
@@ -4097,7 +4106,7 @@
         <v>46256.0</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="F11" s="2">
         <v>1.0</v>
@@ -4117,10 +4126,10 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>66</v>
@@ -4129,7 +4138,7 @@
         <v>46256.0</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="F12" s="2">
         <v>1.0</v>
@@ -4149,10 +4158,10 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>66</v>
@@ -4161,7 +4170,7 @@
         <v>46256.0</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="F13" s="2">
         <v>1.0</v>
@@ -4181,10 +4190,10 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>66</v>
@@ -4193,7 +4202,7 @@
         <v>46256.0</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="F14" s="2">
         <v>1.0</v>
@@ -4213,10 +4222,10 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>66</v>
@@ -4225,7 +4234,7 @@
         <v>46256.0</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="F15" s="2">
         <v>3.5</v>
@@ -4245,10 +4254,10 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>66</v>
@@ -4257,7 +4266,7 @@
         <v>46256.0</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="F16" s="2">
         <v>3.5</v>
@@ -4277,10 +4286,10 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>66</v>
@@ -4289,7 +4298,7 @@
         <v>46256.0</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="F17" s="2">
         <v>1.0</v>
@@ -4309,10 +4318,10 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>66</v>
@@ -4321,7 +4330,7 @@
         <v>46256.0</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="F18" s="2">
         <v>1.0</v>
@@ -4341,10 +4350,10 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>80</v>
@@ -4353,7 +4362,7 @@
         <v>46256.0</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="F19" s="2">
         <v>90.0</v>
@@ -4373,10 +4382,10 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>80</v>
@@ -4385,7 +4394,7 @@
         <v>46256.0</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="F20" s="2">
         <v>90.0</v>
@@ -4405,10 +4414,10 @@
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>80</v>
@@ -4417,7 +4426,7 @@
         <v>46256.0</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="F21" s="2">
         <v>90.0</v>
@@ -4437,10 +4446,10 @@
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>80</v>
@@ -4449,7 +4458,7 @@
         <v>46256.0</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="F22" s="2">
         <v>90.0</v>
@@ -4469,10 +4478,10 @@
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="2" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>66</v>
@@ -4481,7 +4490,7 @@
         <v>46256.0</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="F23" s="2">
         <v>2.5</v>
@@ -4501,10 +4510,10 @@
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="2" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>66</v>
@@ -4513,7 +4522,7 @@
         <v>46256.0</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="F24" s="2">
         <v>2.5</v>
@@ -4533,10 +4542,10 @@
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="2" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>92</v>
@@ -4545,7 +4554,7 @@
         <v>46256.0</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="F25" s="2">
         <v>1.5</v>
@@ -4565,10 +4574,10 @@
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="2" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>92</v>
@@ -4577,7 +4586,7 @@
         <v>46256.0</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="F26" s="2">
         <v>1.5</v>
@@ -4597,10 +4606,10 @@
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="B27" s="2" t="s">
         <v>192</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>189</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>92</v>
@@ -4609,7 +4618,7 @@
         <v>46256.0</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="F27" s="2">
         <v>1.5</v>
@@ -4629,10 +4638,10 @@
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="2" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>100</v>
@@ -4641,7 +4650,7 @@
         <v>46256.0</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="F28" s="2">
         <v>45.0</v>
@@ -4661,10 +4670,10 @@
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="2" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>100</v>
@@ -4673,7 +4682,7 @@
         <v>46256.0</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="F29" s="2">
         <v>30.0</v>
@@ -4693,10 +4702,10 @@
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="2" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>117</v>
@@ -4705,7 +4714,7 @@
         <v>46253.0</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="F30" s="2">
         <v>68.2</v>
@@ -4725,16 +4734,16 @@
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="2" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>133</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="F31" s="2">
         <v>22.22222222222222</v>
@@ -4754,16 +4763,16 @@
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="B32" s="2" t="s">
         <v>200</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>197</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>133</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="F32" s="2">
         <v>81.30081300813008</v>
@@ -5771,19 +5780,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="2">
@@ -5791,7 +5800,7 @@
         <v>19</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="D2" s="2">
         <v>1.0</v>
@@ -5805,7 +5814,7 @@
         <v>26</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="D3" s="2">
         <v>1.0</v>
@@ -5819,7 +5828,7 @@
         <v>34</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="D4" s="2">
         <v>1.0</v>
@@ -5833,7 +5842,7 @@
         <v>48</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="D5" s="2">
         <v>1.0</v>
@@ -5847,7 +5856,7 @@
         <v>61</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="D6" s="2">
         <v>1.0</v>
@@ -5861,7 +5870,7 @@
         <v>71</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="D7" s="2">
         <v>1.0</v>
@@ -5875,7 +5884,7 @@
         <v>86</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="D8" s="2">
         <v>1.0</v>
@@ -5889,7 +5898,7 @@
         <v>97</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="D9" s="2">
         <v>1.0</v>
@@ -5903,7 +5912,7 @@
         <v>101</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="D10" s="2">
         <v>1.0</v>
@@ -5917,7 +5926,7 @@
         <v>110</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="D11" s="2">
         <v>1.0</v>
@@ -5931,7 +5940,7 @@
         <v>110</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="D12" s="2">
         <v>1.0</v>
@@ -6942,34 +6951,34 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
     </row>
     <row r="2">
@@ -6977,7 +6986,7 @@
         <v>1.0</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="C2" s="2">
         <v>250.0</v>
@@ -6997,7 +7006,7 @@
         <v>2.0</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="C3" s="2">
         <v>1800.0</v>
@@ -7014,7 +7023,7 @@
         <v>3.0</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="C4" s="2">
         <v>1155.0</v>
@@ -7034,7 +7043,7 @@
         <v>4.0</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="C5" s="2">
         <v>999.0</v>
@@ -7051,7 +7060,7 @@
         <v>5.0</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="C6" s="2">
         <v>468.65</v>
@@ -7068,7 +7077,7 @@
         <v>6.0</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="C7" s="2">
         <v>2898.24</v>
@@ -7088,7 +7097,7 @@
         <v>7.0</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="C8" s="2">
         <v>2670.0</v>
@@ -7108,7 +7117,7 @@
         <v>8.0</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="C9" s="2">
         <v>438.0</v>
@@ -7125,7 +7134,7 @@
         <v>9.0</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="C10" s="2">
         <v>420.4</v>
@@ -7142,7 +7151,7 @@
         <v>10.0</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="C11" s="2">
         <v>200.0</v>
@@ -7159,7 +7168,7 @@
         <v>11.0</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="C12" s="4">
         <v>892.5</v>
@@ -7179,7 +7188,7 @@
         <v>12.0</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="C13" s="2">
         <v>470.0</v>
@@ -7196,7 +7205,7 @@
         <v>13.0</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="C14" s="2">
         <v>400.0</v>
@@ -7216,7 +7225,7 @@
         <v>14.0</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="C15" s="2">
         <v>594.0</v>
@@ -7236,7 +7245,7 @@
         <v>15.0</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="C16" s="2">
         <v>371.35</v>
@@ -7253,7 +7262,7 @@
         <v>16.0</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="C17" s="2">
         <v>572.0</v>
@@ -7273,7 +7282,7 @@
         <v>17.0</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="C18" s="2">
         <v>468.0</v>
@@ -7293,7 +7302,7 @@
         <v>18.0</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="C19" s="2">
         <v>813.27</v>
@@ -8308,19 +8317,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -9323,15 +9332,15 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="B3" s="2">
         <v>38154.148</v>
@@ -9339,7 +9348,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="B4" s="2">
         <v>34.0</v>
@@ -9347,7 +9356,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="B5" s="2">
         <v>18.0</v>
@@ -9355,7 +9364,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="B6" s="2">
         <v>6402.0</v>
@@ -9363,7 +9372,7 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="B7" s="2">
         <v>44556.148</v>
@@ -9371,7 +9380,7 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="B8" s="2">
         <v>18060.0</v>
@@ -9379,7 +9388,7 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="B9" s="2">
         <v>0.0</v>
@@ -9387,7 +9396,7 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="B10" s="2">
         <v>69018.148</v>
@@ -10393,22 +10402,22 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>

</xml_diff>